<commit_message>
update office IP + telegram test account
</commit_message>
<xml_diff>
--- a/forms/GoldenBounty_PG_NewCurrency_USD_Production.xlsx
+++ b/forms/GoldenBounty_PG_NewCurrency_USD_Production.xlsx
@@ -2545,7 +2545,7 @@
       <c r="C35" s="114" t="n"/>
       <c r="D35" s="11" t="inlineStr">
         <is>
-          <t>37.111.223.255</t>
+          <t>31.59.20.176</t>
         </is>
       </c>
       <c r="E35" s="11" t="inlineStr">
@@ -3298,7 +3298,7 @@
       <c r="C50" s="114" t="n"/>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>37.111.223.255</t>
+          <t>31.59.20.176</t>
         </is>
       </c>
       <c r="E50" s="11" t="inlineStr">
@@ -30889,7 +30889,7 @@
       </c>
       <c r="D18" s="45" t="inlineStr">
         <is>
-          <t>Test account: pgtest@golden-bounty.com (email login enabled for PG QA). Password will be provided to PG Support separately. Open https://golden-bounty.com/login — full access to all games, deposit, withdraw and wallet.</t>
+          <t>Login is via Telegram Mini App (Telegram-based authentication only; no email/password and no Google login). Test account — Telegram username: @golden_bounty_tg, Telegram ID: 8802067922. Open the app from Telegram: https://t.me/golden_bounty_tg — this account has access to all games, deposit, withdraw and wallet functions.</t>
         </is>
       </c>
     </row>

</xml_diff>